<commit_message>
Añade TerriTek, ProcediTek y SosteniTek ESG; quita SimVenture
- Contaduría Pública: TerriTek en Tributaria II, ProcediTek en Derecho
  Aduanero y Fiscal y SosteniTek ESG en Sostenibilidad y Empresa, los
  tres como encaje parcial y validados contra sus repositorios.
- SimVenture Evolution y Validate salen del deck y del Excel.
- Deck y Excel coinciden: 114 asignaturas (79 de aplicación directa,
  35 como apoyo al curso) y 28 simuladores.
- Ficha de Marketing: se quita «el programa con mayor variedad», que
  no era cierto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Universidad El Bosque - CG + otros simuladores SNC.xlsx
+++ b/Universidad El Bosque - CG + otros simuladores SNC.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5786" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5783" uniqueCount="489">
   <si>
     <t>Negocios Internacionales · Presencial</t>
   </si>
@@ -692,10 +692,10 @@
     <t>· Se agregó un bloque nuevo (columnas I–M en cada hoja de programa e I–N en este resumen) con los demás</t>
   </si>
   <si>
-    <t xml:space="preserve">  simuladores de Simuladores de Negocios Colombia: SimVenture Evolution, SimVenture Validate, SimProject,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  SimAgile y los nuevos desarrollos Auditek y RentaSim (ver hoja 'Catálogo otros SNC'). Las columnas A–H</t>
+    <t xml:space="preserve">  simuladores de Simuladores de Negocios Colombia: SimProject, SimAgile y los nuevos desarrollos de la</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  línea PraxiLab (RentaSim, TerriTek, ProcediTek, Auditek y SosteniTek ESG; ver hoja 'Catálogo otros SNC'). Las columnas A–H</t>
   </si>
   <si>
     <t xml:space="preserve">  originales (mapeo CompanyGame, grados de ajuste y recomendaciones) no se modificaron.</t>
@@ -707,15 +707,15 @@
     <t>· Se mantuvo la regla del proyecto: un mismo simulador no se repite en más de una materia por programa;</t>
   </si>
   <si>
-    <t xml:space="preserve">  se priorizaron materias sin encaje CG y, cuando no había, se usó como complemento (p. ej. Validate en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Emprendimiento junto a Fitness Gym). En Project Management se proponen SimProject + SimAgile juntos</t>
+    <t xml:space="preserve">  se priorizaron materias sin encaje CG. En Project Management se proponen SimProject + SimAgile juntos</t>
   </si>
   <si>
     <t xml:space="preserve">  (enfoque predictivo y ágil).</t>
   </si>
   <si>
+    <t xml:space="preserve">  Simuladores de la línea PraxiLab validados contra sus repositorios en octubre de 2026.</t>
+  </si>
+  <si>
     <t>· Auditek y RentaSim se ubicaron donde ya estaban anotados en Contaduría (Revisoría Fiscal y Tributaria I),</t>
   </si>
   <si>
@@ -1461,6 +1461,57 @@
   </si>
   <si>
     <t>Negocios Internacionales · Virtual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SosteniTek ESG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SosteniTek ESG (materialidad, reporte de sostenibilidad y aseguramiento no financiero) con el alcance «Solo matriz» que su spec prevé para cuando la sostenibilidad es un módulo dentro de otra asignatura. Cubre materialidad y reporte; no el resto de la asignatura. Validado contra el repositorio praxilab/sostenitek (oct-2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TerriTek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TerriTek (ICA, reteICA, avisos y tableros, sobretasas): su spec lo ubica en «Tributaria II» / impuestos territoriales. Cubre la parte territorial; no el resto de la asignatura (p. ej. IVA). Validado contra el repositorio praxilab/territek (oct-2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ProcediTek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ProcediTek (requerimiento especial, liquidación oficial de revisión y recurso de reconsideración, en firma de 3-4 estudiantes): pensado para Procedimiento Tributario. Cubre el componente fiscal; no el aduanero. Validado contra el repositorio praxilab/proceditek (oct-2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulador del ciclo tributario territorial (nuevo desarrollo, línea PraxiLab de Grupo Edutec): ICA, reteICA (ambas caras), avisos y tableros y sobretasas. Individual; el estudiante resuelve en qué municipio y cuánto tributa cada operación, defiende la matriz ante las objeciones del municipio y escribe la carta al gerente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tributaria II / Tributaria territorial, Impuestos territoriales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validado contra el repositorio praxilab/territek (oct-2026). Spec v1.1 pendiente de validación tributaria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulador de procedimiento tributario y defensa ante la administración (nuevo desarrollo, línea PraxiLab de Grupo Edutec). Grupal, 3-4 estudiantes con roles en una firma: requerimiento especial de la DIAN, liquidación oficial de revisión y recurso de reconsideración, con control de términos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obligaciones y Procedimiento Tributario, Derecho Fiscal / Procedimiento tributario.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validado contra el repositorio praxilab/proceditek (oct-2026). Catálogo con validación provisional; revisión profesional pendiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulador de materialidad, reporte de sostenibilidad y aseguramiento no financiero (nuevo desarrollo, línea PraxiLab de Grupo Edutec). Individual; el estudiante decide qué asuntos son materiales y si el dato no financiero es aseverable. Alcance configurable: solo matriz, matriz + revelación o ciclo completo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reportes integrados, Contabilidad ambiental, Informes de sostenibilidad, Sostenibilidad y empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validado contra el repositorio praxilab/sostenitek (oct-2026). Solo el caso A está completo; contenido normativo pendiente de validación experta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validado contra el repositorio praxilab/auditek (oct-2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validado contra el repositorio paula-praxilab/rentasim-presentacion (oct-2026).</t>
   </si>
 </sst>
 </file>
@@ -2615,7 +2666,7 @@
       </c>
       <c r="J7" s="35">
         <f>COUNTIF('Adm. Empresas (Presencial)'!$K$3:$K$200,"Encaje parcial")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="35">
         <f>COUNTIF('Adm. Empresas (Presencial)'!$M$3:$M$200,"Encaje perfecto")</f>
@@ -2664,7 +2715,7 @@
       </c>
       <c r="J8" s="35">
         <f>COUNTIF('Adm. Empresas (Virtual)'!$K$3:$K$200,"Encaje parcial")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="35">
         <f>COUNTIF('Adm. Empresas (Virtual)'!$M$3:$M$200,"Encaje perfecto")</f>
@@ -2713,7 +2764,7 @@
       </c>
       <c r="J9" s="35">
         <f>COUNTIF('Adm. Producción y Logística'!$K$3:$K$200,"Encaje parcial")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="35">
         <f>COUNTIF('Adm. Producción y Logística'!$M$3:$M$200,"Encaje perfecto")</f>
@@ -2758,15 +2809,15 @@
       </c>
       <c r="I10" s="35">
         <f>COUNTIF('Adm. Negocios Sostenibles'!$K$3:$K$200,"Encaje perfecto")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="35">
         <f>COUNTIF('Adm. Negocios Sostenibles'!$K$3:$K$200,"Encaje parcial")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="35">
         <f>COUNTIF('Adm. Negocios Sostenibles'!$M$3:$M$200,"Encaje perfecto")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L10" s="35">
         <f>COUNTIF('Adm. Negocios Sostenibles'!$M$3:$M$200,"Encaje parcial")</f>
@@ -2774,11 +2825,11 @@
       </c>
       <c r="M10" s="36">
         <f t="shared" si="1"/>
-        <v>0.16666666666666666</v>
+        <v>0.15151515151515152</v>
       </c>
       <c r="N10" s="37">
         <f t="shared" si="2"/>
-        <v>3.0303030303030303</v>
+        <v>1.5151515151515165</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.25">
@@ -2811,7 +2862,7 @@
       </c>
       <c r="J11" s="35">
         <f>COUNTIF('Contaduría Pública'!$K$3:$K$200,"Encaje parcial")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" s="35">
         <f>COUNTIF('Contaduría Pública'!$M$3:$M$200,"Encaje perfecto")</f>
@@ -2819,15 +2870,15 @@
       </c>
       <c r="L11" s="35">
         <f>COUNTIF('Contaduría Pública'!$M$3:$M$200,"Encaje parcial")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M11" s="36">
         <f t="shared" si="1"/>
-        <v>0.15151515151515152</v>
+        <v>0.19696969696969696</v>
       </c>
       <c r="N11" s="37">
         <f t="shared" si="2"/>
-        <v>3.0303030303030303</v>
+        <v>7.575757575757574</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
@@ -2860,7 +2911,7 @@
       </c>
       <c r="J12" s="35">
         <f>COUNTIF(Economía!$K$3:$K$200,"Encaje parcial")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="35">
         <f>COUNTIF(Economía!$M$3:$M$200,"Encaje perfecto")</f>
@@ -2909,7 +2960,7 @@
       </c>
       <c r="J13" s="35">
         <f>COUNTIF(Finanzas!$K$3:$K$200,"Encaje parcial")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="35">
         <f>COUNTIF(Finanzas!$M$3:$M$200,"Encaje perfecto")</f>
@@ -2954,7 +3005,7 @@
       </c>
       <c r="I14" s="35">
         <f>COUNTIF('Marketing y Transf. Digital'!$K$3:$K$200,"Encaje perfecto")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="35">
         <f>COUNTIF('Marketing y Transf. Digital'!$K$3:$K$200,"Encaje parcial")</f>
@@ -2962,7 +3013,7 @@
       </c>
       <c r="K14" s="35">
         <f>COUNTIF('Marketing y Transf. Digital'!$M$3:$M$200,"Encaje perfecto")</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L14" s="35">
         <f>COUNTIF('Marketing y Transf. Digital'!$M$3:$M$200,"Encaje parcial")</f>
@@ -2970,11 +3021,11 @@
       </c>
       <c r="M14" s="36">
         <f t="shared" si="1"/>
-        <v>0.21212121212121213</v>
+        <v>0.19696969696969696</v>
       </c>
       <c r="N14" s="37">
         <f t="shared" si="2"/>
-        <v>3.0303030303030303</v>
+        <v>1.5151515151515138</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.25">
@@ -3007,7 +3058,7 @@
       </c>
       <c r="J15" s="35">
         <f>COUNTIF('Negocios Internac. (Presenc.)'!$K$3:$K$200,"Encaje parcial")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K15" s="35">
         <f>COUNTIF('Negocios Internac. (Presenc.)'!$M$3:$M$200,"Encaje perfecto")</f>
@@ -3015,15 +3066,15 @@
       </c>
       <c r="L15" s="35">
         <f>COUNTIF('Negocios Internac. (Presenc.)'!$M$3:$M$200,"Encaje parcial")</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M15" s="36">
         <f t="shared" si="1"/>
-        <v>0.234375</v>
+        <v>0.203125</v>
       </c>
       <c r="N15" s="37">
         <f t="shared" si="2"/>
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
@@ -3056,7 +3107,7 @@
       </c>
       <c r="J16" s="35">
         <f>COUNTIF('Negocios Internac. (Virtual)'!$K$3:$K$200,"Encaje parcial")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K16" s="35">
         <f>COUNTIF('Negocios Internac. (Virtual)'!$M$3:$M$200,"Encaje perfecto")</f>
@@ -3064,15 +3115,15 @@
       </c>
       <c r="L16" s="35">
         <f>COUNTIF('Negocios Internac. (Virtual)'!$M$3:$M$200,"Encaje parcial")</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M16" s="36">
         <f t="shared" si="1"/>
-        <v>0.234375</v>
+        <v>0.203125</v>
       </c>
       <c r="N16" s="37">
         <f t="shared" si="2"/>
-        <v>4.6875</v>
+        <v>1.5625</v>
       </c>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
@@ -3101,27 +3152,27 @@
       </c>
       <c r="I17" s="38">
         <f>SUM(I7:I16)</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J17" s="38">
         <f>SUM(J7:J16)</f>
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="K17" s="38">
         <f>SUM(K7:K16)</f>
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L17" s="38">
         <f>SUM(L7:L16)</f>
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M17" s="39">
         <f t="shared" si="1"/>
-        <v>0.17889908256880735</v>
+        <v>0.1743119266055046</v>
       </c>
       <c r="N17" s="40">
         <f t="shared" si="2"/>
-        <v>2.4464831804281357</v>
+        <v>1.9877675840978604</v>
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
@@ -5070,18 +5121,16 @@
       </c>
       <c r="G44" s="26"/>
       <c r="H44" s="23"/>
-      <c r="I44" s="45" t="s">
-        <v>102</v>
+      <c r="I44" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J44" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K44" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L44" s="47" t="s">
-        <v>416</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K44" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L44" s="47"/>
       <c r="M44" s="35" t="str">
         <f t="shared" si="1"/>
         <v>Encaje parcial</v>
@@ -7082,21 +7131,19 @@
       </c>
       <c r="G31" s="26"/>
       <c r="H31" s="23"/>
-      <c r="I31" s="45" t="s">
-        <v>102</v>
+      <c r="I31" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J31" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K31" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="L31" s="47" t="s">
-        <v>457</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K31" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" s="47"/>
       <c r="M31" s="35" t="str">
         <f t="shared" si="0"/>
-        <v>Encaje perfecto</v>
+        <v>No encaja</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
@@ -10118,21 +10165,19 @@
       </c>
       <c r="G46" s="26"/>
       <c r="H46" s="23"/>
-      <c r="I46" s="45" t="s">
-        <v>96</v>
+      <c r="I46" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J46" s="35" t="s">
-        <v>97</v>
-      </c>
-      <c r="K46" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L46" s="47" t="s">
-        <v>98</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K46" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L46" s="47"/>
       <c r="M46" s="35" t="str">
         <f t="shared" si="1"/>
-        <v>Encaje parcial</v>
+        <v>No encaja</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
@@ -10192,21 +10237,19 @@
       </c>
       <c r="G48" s="26"/>
       <c r="H48" s="23"/>
-      <c r="I48" s="45" t="s">
-        <v>102</v>
+      <c r="I48" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J48" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K48" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L48" s="47" t="s">
-        <v>104</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K48" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L48" s="47"/>
       <c r="M48" s="35" t="str">
         <f t="shared" si="1"/>
-        <v>Encaje parcial</v>
+        <v>No encaja</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
@@ -12538,21 +12581,19 @@
       </c>
       <c r="G46" s="26"/>
       <c r="H46" s="23"/>
-      <c r="I46" s="45" t="s">
-        <v>96</v>
+      <c r="I46" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J46" s="35" t="s">
-        <v>97</v>
-      </c>
-      <c r="K46" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L46" s="47" t="s">
-        <v>98</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K46" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L46" s="47"/>
       <c r="M46" s="35" t="str">
         <f t="shared" si="1"/>
-        <v>Encaje parcial</v>
+        <v>No encaja</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
@@ -12612,21 +12653,19 @@
       </c>
       <c r="G48" s="26"/>
       <c r="H48" s="23"/>
-      <c r="I48" s="45" t="s">
-        <v>102</v>
+      <c r="I48" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J48" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K48" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L48" s="47" t="s">
-        <v>104</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K48" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L48" s="47"/>
       <c r="M48" s="35" t="str">
         <f t="shared" si="1"/>
-        <v>Encaje parcial</v>
+        <v>No encaja</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
@@ -13862,7 +13901,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A2:F10"/>
+  <dimension ref="A2:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -13902,104 +13941,104 @@
         <v>316</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A5" s="44" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="B5" s="45" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="D5" s="46" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="E5" s="46" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="F5" s="46" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="44" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>102</v>
+        <v>327</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="D6" s="46" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="44" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B7" s="45" t="s">
-        <v>83</v>
+        <v>331</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>84</v>
+        <v>332</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="E7" s="46" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="F7" s="46" t="s">
-        <v>326</v>
+        <v>487</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="44" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>84</v>
+        <v>332</v>
       </c>
       <c r="D8" s="46" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="E8" s="46" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="F8" s="46" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="44" t="s">
         <v>330</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>331</v>
+        <v>474</v>
       </c>
       <c r="C9" s="35" t="s">
         <v>332</v>
       </c>
       <c r="D9" s="46" t="s">
-        <v>333</v>
+        <v>478</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>334</v>
+        <v>479</v>
       </c>
       <c r="F9" s="46" t="s">
-        <v>335</v>
+        <v>480</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
@@ -14007,19 +14046,39 @@
         <v>330</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>336</v>
+        <v>476</v>
       </c>
       <c r="C10" s="35" t="s">
         <v>332</v>
       </c>
       <c r="D10" s="46" t="s">
-        <v>337</v>
+        <v>481</v>
       </c>
       <c r="E10" s="46" t="s">
-        <v>338</v>
+        <v>482</v>
       </c>
       <c r="F10" s="46" t="s">
-        <v>335</v>
+        <v>483</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="44" t="s">
+        <v>330</v>
+      </c>
+      <c r="B11" s="45" t="s">
+        <v>472</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>484</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>485</v>
+      </c>
+      <c r="F11" s="46" t="s">
+        <v>486</v>
       </c>
     </row>
   </sheetData>
@@ -15561,18 +15620,16 @@
       </c>
       <c r="G43" s="26"/>
       <c r="H43" s="23"/>
-      <c r="I43" s="45" t="s">
-        <v>102</v>
+      <c r="I43" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J43" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K43" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L43" s="47" t="s">
-        <v>345</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K43" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L43" s="47"/>
       <c r="M43" s="35" t="str">
         <f>IF(OR(F43="Encaje perfecto",K43="Encaje perfecto"),"Encaje perfecto",IF(OR(F43="Encaje parcial",K43="Encaje parcial"),"Encaje parcial","No encaja"))</f>
         <v>Encaje parcial</v>
@@ -18045,18 +18102,16 @@
       </c>
       <c r="G43" s="26"/>
       <c r="H43" s="23"/>
-      <c r="I43" s="45" t="s">
-        <v>102</v>
+      <c r="I43" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J43" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K43" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L43" s="47" t="s">
-        <v>345</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K43" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L43" s="47"/>
       <c r="M43" s="35" t="str">
         <f t="shared" si="1"/>
         <v>Encaje parcial</v>
@@ -20545,18 +20600,16 @@
       </c>
       <c r="G44" s="26"/>
       <c r="H44" s="23"/>
-      <c r="I44" s="45" t="s">
-        <v>102</v>
+      <c r="I44" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J44" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K44" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L44" s="47" t="s">
-        <v>370</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K44" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L44" s="47"/>
       <c r="M44" s="35" t="str">
         <f t="shared" si="1"/>
         <v>Encaje parcial</v>
@@ -23029,14 +23082,14 @@
       </c>
       <c r="G45" s="26"/>
       <c r="H45" s="23"/>
-      <c r="I45" s="45" t="s">
-        <v>102</v>
+      <c r="I45" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J45" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K45" s="48" t="s">
-        <v>85</v>
+        <v>19</v>
+      </c>
+      <c r="K45" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="L45" s="47"/>
       <c r="M45" s="35" t="str">
@@ -23177,21 +23230,19 @@
       </c>
       <c r="G49" s="26"/>
       <c r="H49" s="23"/>
-      <c r="I49" s="45" t="s">
-        <v>102</v>
+      <c r="I49" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J49" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K49" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="L49" s="47" t="s">
-        <v>397</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K49" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L49" s="47"/>
       <c r="M49" s="35" t="str">
         <f t="shared" si="1"/>
-        <v>Encaje perfecto</v>
+        <v>No encaja</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
@@ -24569,19 +24620,21 @@
       </c>
       <c r="G19" s="26"/>
       <c r="H19" s="23"/>
-      <c r="I19" s="35" t="s">
-        <v>19</v>
+      <c r="I19" s="45" t="s">
+        <v>472</v>
       </c>
       <c r="J19" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="K19" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="L19" s="47"/>
+        <v>332</v>
+      </c>
+      <c r="K19" s="48" t="s">
+        <v>85</v>
+      </c>
+      <c r="L19" s="47" t="s">
+        <v>473</v>
+      </c>
       <c r="M19" s="35" t="str">
         <f t="shared" si="0"/>
-        <v>No encaja</v>
+        <v>Encaje parcial</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -25297,19 +25350,21 @@
       </c>
       <c r="G39" s="26"/>
       <c r="H39" s="23"/>
-      <c r="I39" s="35" t="s">
-        <v>19</v>
+      <c r="I39" s="45" t="s">
+        <v>474</v>
       </c>
       <c r="J39" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="K39" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="L39" s="47"/>
+        <v>332</v>
+      </c>
+      <c r="K39" s="48" t="s">
+        <v>85</v>
+      </c>
+      <c r="L39" s="47" t="s">
+        <v>475</v>
+      </c>
       <c r="M39" s="35" t="str">
         <f t="shared" si="1"/>
-        <v>No encaja</v>
+        <v>Encaje parcial</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
@@ -25477,18 +25532,16 @@
       </c>
       <c r="G44" s="26"/>
       <c r="H44" s="23"/>
-      <c r="I44" s="45" t="s">
-        <v>102</v>
+      <c r="I44" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J44" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K44" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L44" s="47" t="s">
-        <v>416</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K44" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L44" s="47"/>
       <c r="M44" s="35" t="str">
         <f t="shared" si="1"/>
         <v>Encaje parcial</v>
@@ -25627,19 +25680,21 @@
       </c>
       <c r="G48" s="26"/>
       <c r="H48" s="23"/>
-      <c r="I48" s="35" t="s">
-        <v>19</v>
+      <c r="I48" s="45" t="s">
+        <v>476</v>
       </c>
       <c r="J48" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="K48" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="L48" s="47"/>
+        <v>332</v>
+      </c>
+      <c r="K48" s="48" t="s">
+        <v>85</v>
+      </c>
+      <c r="L48" s="47" t="s">
+        <v>477</v>
+      </c>
       <c r="M48" s="35" t="str">
         <f t="shared" si="1"/>
-        <v>No encaja</v>
+        <v>Encaje parcial</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
@@ -27995,18 +28050,16 @@
       </c>
       <c r="G45" s="26"/>
       <c r="H45" s="23"/>
-      <c r="I45" s="45" t="s">
-        <v>102</v>
+      <c r="I45" s="35" t="s">
+        <v>19</v>
       </c>
       <c r="J45" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="K45" s="48" t="s">
-        <v>85</v>
-      </c>
-      <c r="L45" s="47" t="s">
-        <v>416</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K45" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L45" s="47"/>
       <c r="M45" s="35" t="str">
         <f t="shared" si="1"/>
         <v>Encaje parcial</v>

</xml_diff>